<commit_message>
feat: add order unit constraint (O-7) — x_small and x_large each must be multiples of order_unit
- Add 発注単位 column to product_master (required)
- Extract order_unit in _prepare_inputs()
- Add k_small/k_large integer variables in optimize() to enforce
  x_small = k_small * u_p and x_large = k_large * u_p individually
- Update fixtures (sample_dfs, sample_excel, dfs_forcing_trucks, dfs_infeasible)
- Add test_O7_1 and test_O7_2 (TDD: Red→Green)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/InputData2.xlsx
+++ b/data/input/InputData2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="商品マスタ" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="16">
   <si>
     <t xml:space="preserve">商品コード</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t xml:space="preserve">配送費_ケース</t>
+  </si>
+  <si>
+    <t xml:space="preserve">発注単位</t>
   </si>
   <si>
     <t xml:space="preserve">Product1</t>
@@ -434,7 +437,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.41015625" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.99"/>
@@ -456,10 +459,13 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>960</v>
@@ -470,10 +476,13 @@
       <c r="D2" s="1" t="n">
         <v>150</v>
       </c>
+      <c r="E2" s="0" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>1152</v>
@@ -484,10 +493,13 @@
       <c r="D3" s="1" t="n">
         <v>120</v>
       </c>
+      <c r="E3" s="0" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>576</v>
@@ -497,6 +509,9 @@
       </c>
       <c r="D4" s="1" t="n">
         <v>200</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -523,15 +538,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="n">
         <v>50000</v>
@@ -564,21 +579,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>46082</v>
@@ -586,14 +601,16 @@
       <c r="C2" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D2" s="5"/>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E2" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" s="4" t="n">
         <v>46083</v>
@@ -601,14 +618,16 @@
       <c r="C3" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D3" s="5"/>
+      <c r="D3" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E3" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" s="4" t="n">
         <v>46084</v>
@@ -616,14 +635,16 @@
       <c r="C4" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D4" s="5"/>
+      <c r="D4" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E4" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B5" s="4" t="n">
         <v>46085</v>
@@ -638,9 +659,9 @@
         <v>99999</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" s="4" t="n">
         <v>46086</v>
@@ -648,14 +669,16 @@
       <c r="C6" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="5"/>
+      <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" s="4" t="n">
         <v>46087</v>
@@ -663,14 +686,16 @@
       <c r="C7" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D7" s="5"/>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E7" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B8" s="4" t="n">
         <v>46088</v>
@@ -678,14 +703,16 @@
       <c r="C8" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D8" s="5"/>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E8" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" s="4" t="n">
         <v>46089</v>
@@ -693,14 +720,16 @@
       <c r="C9" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D9" s="5"/>
+      <c r="D9" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E9" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>46090</v>
@@ -715,9 +744,9 @@
         <v>99999</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>46091</v>
@@ -725,14 +754,16 @@
       <c r="C11" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D11" s="5"/>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E11" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B12" s="4" t="n">
         <v>46092</v>
@@ -747,9 +778,9 @@
         <v>99999</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>46093</v>
@@ -757,14 +788,16 @@
       <c r="C13" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D13" s="5"/>
+      <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E13" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B14" s="4" t="n">
         <v>46094</v>
@@ -779,9 +812,9 @@
         <v>99999</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="14" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B15" s="4" t="n">
         <v>46095</v>
@@ -789,14 +822,16 @@
       <c r="C15" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D15" s="5"/>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E15" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B16" s="4" t="n">
         <v>46096</v>
@@ -813,7 +848,7 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>46097</v>
@@ -821,14 +856,16 @@
       <c r="C17" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D17" s="5"/>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E17" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>46098</v>
@@ -845,7 +882,7 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B19" s="4" t="n">
         <v>46099</v>
@@ -853,14 +890,16 @@
       <c r="C19" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D19" s="5"/>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E19" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B20" s="4" t="n">
         <v>46100</v>
@@ -877,7 +916,7 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B21" s="4" t="n">
         <v>46101</v>
@@ -885,14 +924,16 @@
       <c r="C21" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D21" s="5"/>
+      <c r="D21" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E21" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B22" s="4" t="n">
         <v>46102</v>
@@ -909,7 +950,7 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B23" s="4" t="n">
         <v>46103</v>
@@ -917,14 +958,16 @@
       <c r="C23" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D23" s="5"/>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E23" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B24" s="4" t="n">
         <v>46104</v>
@@ -941,7 +984,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B25" s="4" t="n">
         <v>46105</v>
@@ -949,14 +992,16 @@
       <c r="C25" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D25" s="5"/>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E25" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B26" s="4" t="n">
         <v>46106</v>
@@ -973,7 +1018,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B27" s="4" t="n">
         <v>46107</v>
@@ -981,14 +1026,16 @@
       <c r="C27" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D27" s="5"/>
+      <c r="D27" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E27" s="5" t="n">
         <v>99999</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B28" s="4" t="n">
         <v>46108</v>
@@ -1005,7 +1052,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B29" s="4" t="n">
         <v>46109</v>
@@ -1013,7 +1060,9 @@
       <c r="C29" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D29" s="5"/>
+      <c r="D29" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="E29" s="5" t="n">
         <v>99999</v>
       </c>
@@ -1042,12 +1091,12 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>500</v>
@@ -1055,7 +1104,7 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>300</v>
@@ -1063,7 +1112,7 @@
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>120</v>

</xml_diff>